<commit_message>
interactive npcs, text boxes
</commit_message>
<xml_diff>
--- a/src/beastmistress/assets/maps/debug.xlsx
+++ b/src/beastmistress/assets/maps/debug.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1822" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1830" uniqueCount="24">
   <si>
     <t>NONE</t>
   </si>
@@ -73,6 +73,21 @@
   </si>
   <si>
     <t>talkingTriggersACutscene?</t>
+  </si>
+  <si>
+    <t>popupTextMessage</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>Talk to Debug NPC (F)</t>
+  </si>
+  <si>
+    <t>whichCutscene?</t>
+  </si>
+  <si>
+    <t>debugNPC1</t>
   </si>
 </sst>
 </file>
@@ -5997,11 +6012,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="15.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="3"/>
+    <col min="1" max="1" width="15.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="3"/>
+    <col min="4" max="4" width="16.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -6102,6 +6120,34 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>